<commit_message>
Updated Auth and Get all IDs
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/AuthData.xlsx
+++ b/src/test/resources/testdata/AuthData.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adhit\OneDrive\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adhit\OneDrive\Desktop\clg\API_testing\sprint\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB41BFCE-A4A2-4C6D-A3DE-E30E63E4EA5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AED039E3-45FF-4392-B93C-E0C5EE44ACFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1565B1A8-1465-4683-98A1-F3CECA7BBA48}"/>
   </bookViews>
   <sheets>
     <sheet name="Auth_data" sheetId="1" r:id="rId1"/>
+    <sheet name="FilterData" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
   <si>
     <t>username</t>
   </si>
@@ -51,6 +52,72 @@
   </si>
   <si>
     <t>admin</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Firstname</t>
+  </si>
+  <si>
+    <t>Lastname</t>
+  </si>
+  <si>
+    <t>Checkin</t>
+  </si>
+  <si>
+    <t>Checkout</t>
+  </si>
+  <si>
+    <t>Adhithya</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Rajmohan</t>
+  </si>
+  <si>
+    <t>T</t>
+  </si>
+  <si>
+    <t>Prithiba</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>Akshaya</t>
+  </si>
+  <si>
+    <t>SK</t>
+  </si>
+  <si>
+    <t>15-03-2001</t>
+  </si>
+  <si>
+    <t>16-03-2001</t>
+  </si>
+  <si>
+    <t>17-03-2001</t>
+  </si>
+  <si>
+    <t>18-03-2001</t>
+  </si>
+  <si>
+    <t>19-03-2001</t>
+  </si>
+  <si>
+    <t>20-03-2001</t>
+  </si>
+  <si>
+    <t>21-03-2001</t>
+  </si>
+  <si>
+    <t>Admin Credentials</t>
   </si>
 </sst>
 </file>
@@ -66,12 +133,30 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -86,8 +171,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -422,7 +517,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6C3887F-1DEF-475D-BDE1-A23E1B73B286}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.21875" customWidth="1"/>
@@ -430,22 +525,130 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
+      <c r="A1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="4"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CB28E0F-3A26-4DA1-9FD3-7C530A677969}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.109375" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="4" width="17.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="3"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>